<commit_message>
Unit root test Exchange rate
</commit_message>
<xml_diff>
--- a/DATA/Aggregated data/Exchange rates/Exchange rates.xlsx
+++ b/DATA/Aggregated data/Exchange rates/Exchange rates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\Desktop\Masterproef\DATA\Aggregated data\Exchange rates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\Documents\GitHub\Masterthesis\DATA\Aggregated data\Exchange rates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07A4E754-55FA-4463-BA76-6B4E94FAA0B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77810A2F-E0EF-4260-BFD0-210780E76286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exchange rates" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="5">
   <si>
     <t>Philippines</t>
   </si>
@@ -53,21 +53,6 @@
   </si>
   <si>
     <t>Korea</t>
-  </si>
-  <si>
-    <t>Min</t>
-  </si>
-  <si>
-    <t>Max</t>
-  </si>
-  <si>
-    <t>Mean</t>
-  </si>
-  <si>
-    <t>Std dev</t>
-  </si>
-  <si>
-    <t>CV</t>
   </si>
 </sst>
 </file>
@@ -8786,18 +8771,6 @@
       <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="K1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L1" t="s">
-        <v>0</v>
-      </c>
-      <c r="M1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N1" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
@@ -8818,25 +8791,10 @@
       <c r="F2" s="3">
         <v>1089.1818181818201</v>
       </c>
-      <c r="J2" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" s="4">
-        <f>MIN(C2:C130)</f>
-        <v>12572.772727272701</v>
-      </c>
-      <c r="L2" s="4">
-        <f t="shared" ref="L2:N2" si="0">MIN(D2:D130)</f>
-        <v>44.130626654898499</v>
-      </c>
-      <c r="M2" s="4">
-        <f t="shared" si="0"/>
-        <v>104.98</v>
-      </c>
-      <c r="N2" s="4">
-        <f t="shared" si="0"/>
-        <v>1066.8869565217401</v>
-      </c>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3">
@@ -8857,25 +8815,10 @@
       <c r="F3" s="3">
         <v>1099.0150000000001</v>
       </c>
-      <c r="J3" t="s">
-        <v>6</v>
-      </c>
-      <c r="K3" s="4">
-        <f>MAX(C2:C130)</f>
-        <v>16768.409090909099</v>
-      </c>
-      <c r="L3" s="4">
-        <f t="shared" ref="L3:N3" si="1">MAX(D2:D130)</f>
-        <v>58.771672054069946</v>
-      </c>
-      <c r="M3" s="4">
-        <f t="shared" si="1"/>
-        <v>130.81</v>
-      </c>
-      <c r="N3" s="4">
-        <f t="shared" si="1"/>
-        <v>1457.5952380952399</v>
-      </c>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4">
@@ -8896,25 +8839,10 @@
       <c r="F4" s="3">
         <v>1113.4181818181801</v>
       </c>
-      <c r="J4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="4">
-        <f>AVERAGE(C2:C130)</f>
-        <v>14474.419925019367</v>
-      </c>
-      <c r="L4" s="4">
-        <f t="shared" ref="L4:N4" si="2">AVERAGE(D2:D130)</f>
-        <v>51.867248965616938</v>
-      </c>
-      <c r="M4" s="4">
-        <f t="shared" si="2"/>
-        <v>116.91689922480617</v>
-      </c>
-      <c r="N4" s="4">
-        <f t="shared" si="2"/>
-        <v>1212.3930287216278</v>
-      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
@@ -8935,25 +8863,6 @@
       <c r="F5" s="3">
         <v>1087.1136363636399</v>
       </c>
-      <c r="J5" t="s">
-        <v>8</v>
-      </c>
-      <c r="K5">
-        <f>_xlfn.STDEV.S(C2:C130)</f>
-        <v>1003.7233842531765</v>
-      </c>
-      <c r="L5">
-        <f t="shared" ref="L5:N5" si="3">_xlfn.STDEV.S(D2:D130)</f>
-        <v>3.8802951940827346</v>
-      </c>
-      <c r="M5">
-        <f t="shared" si="3"/>
-        <v>6.6764072484815911</v>
-      </c>
-      <c r="N5">
-        <f t="shared" si="3"/>
-        <v>105.56471811888797</v>
-      </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
@@ -8973,25 +8882,6 @@
       </c>
       <c r="F6" s="3">
         <v>1091.5142857142901</v>
-      </c>
-      <c r="J6" t="s">
-        <v>9</v>
-      </c>
-      <c r="K6">
-        <f>K5/K4</f>
-        <v>6.9344636223951026E-2</v>
-      </c>
-      <c r="L6">
-        <f t="shared" ref="L6:N6" si="4">L5/L4</f>
-        <v>7.4812049442896073E-2</v>
-      </c>
-      <c r="M6">
-        <f t="shared" si="4"/>
-        <v>5.7103868583140309E-2</v>
-      </c>
-      <c r="N6">
-        <f t="shared" si="4"/>
-        <v>8.7071366807674216E-2</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -11484,14 +11374,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB0B114D-209E-4B95-A185-D88DBA8646B9}">
-  <dimension ref="B1:Y130"/>
+  <dimension ref="B1:F130"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>1</v>
       </c>
@@ -11508,7 +11398,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" s="1">
         <v>42005</v>
       </c>
@@ -11528,20 +11418,8 @@
         <f>'Exchange rates'!F2/'Exchange rates'!F$2</f>
         <v>1</v>
       </c>
-      <c r="V2" t="s">
-        <v>2</v>
-      </c>
-      <c r="W2" t="s">
-        <v>0</v>
-      </c>
-      <c r="X2" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="2:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="1">
         <v>42036</v>
       </c>
@@ -11561,27 +11439,8 @@
         <f>'Exchange rates'!F3/'Exchange rates'!F$2</f>
         <v>1.0090280444036375</v>
       </c>
-      <c r="U3" t="s">
-        <v>5</v>
-      </c>
-      <c r="V3">
-        <f>MIN(C2:C130)</f>
-        <v>1</v>
-      </c>
-      <c r="W3">
-        <f t="shared" ref="W3:Y3" si="0">MIN(D2:D130)</f>
-        <v>0.9975286849073256</v>
-      </c>
-      <c r="X3">
-        <f t="shared" si="0"/>
-        <v>0.95150910903652686</v>
-      </c>
-      <c r="Y3">
-        <f t="shared" si="0"/>
-        <v>0.97953063364820303</v>
-      </c>
-    </row>
-    <row r="4" spans="2:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="1">
         <v>42064</v>
       </c>
@@ -11601,27 +11460,8 @@
         <f>'Exchange rates'!F4/'Exchange rates'!F$2</f>
         <v>1.0222518988398264</v>
       </c>
-      <c r="U4" t="s">
-        <v>6</v>
-      </c>
-      <c r="V4">
-        <f>MAX(C2:C130)</f>
-        <v>1.3337081210841644</v>
-      </c>
-      <c r="W4">
-        <f t="shared" ref="W4:Y4" si="1">MAX(D2:D130)</f>
-        <v>1.3284748751101969</v>
-      </c>
-      <c r="X4">
-        <f t="shared" si="1"/>
-        <v>1.1856249433517629</v>
-      </c>
-      <c r="Y4">
-        <f t="shared" si="1"/>
-        <v>1.3382478607000761</v>
-      </c>
-    </row>
-    <row r="5" spans="2:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <v>42095</v>
       </c>
@@ -11641,27 +11481,8 @@
         <f>'Exchange rates'!F5/'Exchange rates'!F$2</f>
         <v>0.99810116017027106</v>
       </c>
-      <c r="U5" t="s">
-        <v>7</v>
-      </c>
-      <c r="V5">
-        <f>AVERAGE(C2:C130)</f>
-        <v>1.1512512187245405</v>
-      </c>
-      <c r="W5">
-        <f t="shared" ref="W5:Y5" si="2">AVERAGE(D2:D130)</f>
-        <v>1.1724072956188059</v>
-      </c>
-      <c r="X5">
-        <f t="shared" si="2"/>
-        <v>1.0597017966537319</v>
-      </c>
-      <c r="Y5">
-        <f t="shared" si="2"/>
-        <v>1.1131227206358303</v>
-      </c>
-    </row>
-    <row r="6" spans="2:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="1">
         <v>42125</v>
       </c>
@@ -11681,27 +11502,8 @@
         <f>'Exchange rates'!F6/'Exchange rates'!F$2</f>
         <v>1.002141485924144</v>
       </c>
-      <c r="U6" t="s">
-        <v>8</v>
-      </c>
-      <c r="V6">
-        <f>_xlfn.STDEV.S(C2:C130)</f>
-        <v>7.9833096964833566E-2</v>
-      </c>
-      <c r="W6">
-        <f t="shared" ref="W6:Y6" si="3">_xlfn.STDEV.S(D2:D130)</f>
-        <v>8.7710192567046139E-2</v>
-      </c>
-      <c r="X6">
-        <f t="shared" si="3"/>
-        <v>6.051307213343235E-2</v>
-      </c>
-      <c r="Y6">
-        <f t="shared" si="3"/>
-        <v>9.6921116710438654E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="2:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <v>42156</v>
       </c>
@@ -11721,27 +11523,8 @@
         <f>'Exchange rates'!F7/'Exchange rates'!F$2</f>
         <v>1.0215758283949588</v>
       </c>
-      <c r="U7" t="s">
-        <v>9</v>
-      </c>
-      <c r="V7">
-        <f>V6+V5</f>
-        <v>1.231084315689374</v>
-      </c>
-      <c r="W7">
-        <f t="shared" ref="W7:Y7" si="4">W6+W5</f>
-        <v>1.2601174881858519</v>
-      </c>
-      <c r="X7">
-        <f t="shared" si="4"/>
-        <v>1.1202148687871643</v>
-      </c>
-      <c r="Y7">
-        <f t="shared" si="4"/>
-        <v>1.210043837346269</v>
-      </c>
-    </row>
-    <row r="8" spans="2:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="1">
         <v>42186</v>
       </c>
@@ -11762,7 +11545,7 @@
         <v>1.0515032859999371</v>
       </c>
     </row>
-    <row r="9" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <v>42217</v>
       </c>
@@ -11783,7 +11566,7 @@
         <v>1.0829360773605849</v>
       </c>
     </row>
-    <row r="10" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="1">
         <v>42248</v>
       </c>
@@ -11804,7 +11587,7 @@
         <v>1.0888698773057297</v>
       </c>
     </row>
-    <row r="11" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="1">
         <v>42278</v>
       </c>
@@ -11825,7 +11608,7 @@
         <v>1.0524747516901709</v>
       </c>
     </row>
-    <row r="12" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="1">
         <v>42309</v>
       </c>
@@ -11846,7 +11629,7 @@
         <v>1.058479099844593</v>
       </c>
     </row>
-    <row r="13" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <v>42339</v>
       </c>
@@ -11867,7 +11650,7 @@
         <v>1.0767755467896643</v>
       </c>
     </row>
-    <row r="14" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="1">
         <v>42370</v>
       </c>
@@ -11888,7 +11671,7 @@
         <v>1.1034713693506741</v>
       </c>
     </row>
-    <row r="15" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" s="1">
         <v>42401</v>
       </c>
@@ -11909,7 +11692,7 @@
         <v>1.1162725903315156</v>
       </c>
     </row>
-    <row r="16" spans="2:25" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="1">
         <v>42430</v>
       </c>

</xml_diff>